<commit_message>
#3 Deliverable Files Added
</commit_message>
<xml_diff>
--- a/Design Files/Bento Pad Mini-v1.0/BOM/Bento Pad Mini-v1.0.xlsx
+++ b/Design Files/Bento Pad Mini-v1.0/BOM/Bento Pad Mini-v1.0.xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="182">
   <si>
     <t>#</t>
   </si>
@@ -156,15 +156,12 @@
     <t>R3, R4</t>
   </si>
   <si>
-    <t>R5</t>
+    <t>R5, R7</t>
   </si>
   <si>
     <t>R6, R8, R9, R10, R11, R12, R14, R15, R16, R17, R18, R19</t>
   </si>
   <si>
-    <t>R7</t>
-  </si>
-  <si>
     <t>R13</t>
   </si>
   <si>
@@ -267,15 +264,12 @@
     <t>RES 5.1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES SMD 1M OHM 5% 1/16W 0402</t>
+    <t>RES SMD 1M OHM 5% 1/16W 0402, RES 1M OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES 10K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES 1M OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
     <t>11mm Encoder with 24 Detent Force 20mm Metal Flatted Shaft PC Pin Horizontal/Rear Facing</t>
   </si>
   <si>
@@ -435,15 +429,12 @@
     <t>RC0402FR-075K1L</t>
   </si>
   <si>
-    <t>AF0402JR-071ML</t>
+    <t>AF0402JR-071ML, RC0402FR-071ML</t>
   </si>
   <si>
     <t>RC0402FR-0710KL</t>
   </si>
   <si>
-    <t>RC0402FR-071ML</t>
-  </si>
-  <si>
     <t>RC0603FR-07499RL</t>
   </si>
   <si>
@@ -567,19 +558,19 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>DO NOT PLACE</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>DO NOT PLACE</t>
-  </si>
-  <si>
-    <t>Custom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -624,7 +615,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <b/>
+      <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -632,7 +624,7 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -754,7 +746,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -794,13 +786,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1090,19 +1085,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1130,65 +1125,65 @@
         <v>19</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="11">
+      <c r="B3" s="15">
         <f>ROW(B3) - ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="I3" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="J3" s="15">
+      <c r="E3" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="J3" s="17">
         <v>5</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B38" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B36" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -1198,19 +1193,19 @@
         <v>21</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1230,19 +1225,19 @@
         <v>22</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1262,19 +1257,19 @@
         <v>23</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1294,19 +1289,19 @@
         <v>24</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1326,19 +1321,19 @@
         <v>25</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1358,19 +1353,19 @@
         <v>26</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1390,19 +1385,19 @@
         <v>27</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1422,19 +1417,19 @@
         <v>28</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1454,19 +1449,19 @@
         <v>29</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1486,19 +1481,19 @@
         <v>30</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1518,19 +1513,19 @@
         <v>31</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J14" s="9">
         <v>13</v>
@@ -1550,19 +1545,19 @@
         <v>32</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="J15" s="7">
         <v>5</v>
@@ -1582,19 +1577,19 @@
         <v>33</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -1614,19 +1609,19 @@
         <v>34</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="J17" s="7">
         <v>3</v>
@@ -1646,19 +1641,19 @@
         <v>35</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1671,26 +1666,24 @@
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="13" t="s">
-        <v>6</v>
-      </c>
+      <c r="C19" s="12"/>
       <c r="D19" s="7" t="s">
         <v>36</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>182</v>
+        <v>148</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>181</v>
       </c>
       <c r="J19" s="7">
         <v>2</v>
@@ -1710,19 +1703,19 @@
         <v>37</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1742,19 +1735,19 @@
         <v>38</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1774,19 +1767,19 @@
         <v>39</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -1806,19 +1799,19 @@
         <v>40</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>182</v>
+        <v>150</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>181</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1838,19 +1831,19 @@
         <v>41</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -1870,19 +1863,19 @@
         <v>42</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>182</v>
+        <v>152</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>181</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
@@ -1902,19 +1895,19 @@
         <v>43</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -1934,26 +1927,26 @@
         <v>44</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J27" s="7">
         <v>2</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -1966,22 +1959,22 @@
         <v>45</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="J28" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" s="9"/>
     </row>
@@ -1998,150 +1991,150 @@
         <v>46</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="J29" s="7">
         <v>12</v>
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>47</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>106</v>
+        <v>180</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>48</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>184</v>
+        <v>106</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="12" t="s">
-        <v>13</v>
+      <c r="C32" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>108</v>
+        <v>180</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="J32" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>50</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J33" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
@@ -2152,25 +2145,25 @@
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>51</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>184</v>
+        <v>87</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>109</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>110</v>
+        <v>139</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>182</v>
+        <v>156</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2190,19 +2183,19 @@
         <v>52</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2222,88 +2215,56 @@
         <v>53</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="I36" s="8" t="s">
-        <v>182</v>
+        <v>156</v>
+      </c>
+      <c r="I36" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
       </c>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
         <v>35</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>54</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>113</v>
+        <v>180</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
       </c>
       <c r="K37" s="7"/>
-    </row>
-    <row r="38" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="1"/>
-      <c r="B38" s="11">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="J38" s="9">
-        <v>1</v>
-      </c>
-      <c r="K38" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>